<commit_message>
Toilets list: charge-line totals fixed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
@@ -4752,13 +4752,13 @@
       </c>
       <c r="F12" s="1" t="inlineStr"/>
       <c r="G12" s="1" t="n">
-        <v>121853.86</v>
+        <v>144463.86</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>26355.32</v>
+        <v>37660.32</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>95498.54000000001</v>
+        <v>106803.54</v>
       </c>
       <c r="J12" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Toilets list: labour and transport breakdown by unit type
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 by reference" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 charge lines" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labour &amp; transport breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 charge lines" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -789,7 +790,6 @@
           <t>9 Main Beach Seaside — Mid-South</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -820,9 +820,6 @@
       <c r="M7" t="n">
         <v>0</v>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1132,9 +1129,6 @@
       <c r="M13" t="n">
         <v>0</v>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1182,9 +1176,6 @@
       <c r="M14" t="n">
         <v>0</v>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1232,9 +1223,6 @@
       <c r="M15" t="n">
         <v>0</v>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1282,9 +1270,6 @@
       <c r="M16" t="n">
         <v>0</v>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1394,9 +1379,6 @@
       <c r="M18" t="n">
         <v>0</v>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1444,9 +1426,6 @@
       <c r="M19" t="n">
         <v>0</v>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1494,9 +1473,6 @@
       <c r="M20" t="n">
         <v>0</v>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1602,9 +1578,6 @@
       <c r="M22" t="n">
         <v>0</v>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1652,9 +1625,6 @@
       <c r="M23" t="n">
         <v>0</v>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1702,9 +1672,6 @@
       <c r="M24" t="n">
         <v>0</v>
       </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1752,9 +1719,6 @@
       <c r="M25" t="n">
         <v>0</v>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1802,9 +1766,6 @@
       <c r="M26" t="n">
         <v>0</v>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1852,9 +1813,6 @@
       <c r="M27" t="n">
         <v>0</v>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1960,9 +1918,6 @@
       <c r="M29" t="n">
         <v>0</v>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2010,9 +1965,6 @@
       <c r="M30" t="n">
         <v>0</v>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2060,9 +2012,6 @@
       <c r="M31" t="n">
         <v>0</v>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2110,9 +2059,6 @@
       <c r="M32" t="n">
         <v>0</v>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2160,9 +2106,6 @@
       <c r="M33" t="n">
         <v>0</v>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2210,9 +2153,6 @@
       <c r="M34" t="n">
         <v>0</v>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2260,9 +2200,6 @@
       <c r="M35" t="n">
         <v>0</v>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2310,9 +2247,6 @@
       <c r="M36" t="n">
         <v>0</v>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2360,9 +2294,6 @@
       <c r="M37" t="n">
         <v>2</v>
       </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2410,9 +2341,6 @@
       <c r="M38" t="n">
         <v>0</v>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2460,9 +2388,6 @@
       <c r="M39" t="n">
         <v>0</v>
       </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2510,9 +2435,6 @@
       <c r="M40" t="n">
         <v>0</v>
       </c>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2560,9 +2482,6 @@
       <c r="M41" t="n">
         <v>0</v>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2610,9 +2529,6 @@
       <c r="M42" t="n">
         <v>0</v>
       </c>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2660,9 +2576,6 @@
       <c r="M43" t="n">
         <v>0</v>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2710,9 +2623,6 @@
       <c r="M44" t="n">
         <v>0</v>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2810,9 +2720,6 @@
       <c r="M46" t="n">
         <v>0</v>
       </c>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2860,9 +2767,6 @@
       <c r="M47" t="n">
         <v>0</v>
       </c>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2910,9 +2814,6 @@
       <c r="M48" t="n">
         <v>0</v>
       </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2960,9 +2861,6 @@
       <c r="M49" t="n">
         <v>0</v>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3010,9 +2908,6 @@
       <c r="M50" t="n">
         <v>0</v>
       </c>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3060,9 +2955,6 @@
       <c r="M51" t="n">
         <v>0</v>
       </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3110,9 +3002,6 @@
       <c r="M52" t="n">
         <v>0</v>
       </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3160,9 +3049,6 @@
       <c r="M53" t="n">
         <v>0</v>
       </c>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3210,9 +3096,6 @@
       <c r="M54" t="n">
         <v>0</v>
       </c>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3310,9 +3193,6 @@
       <c r="M56" t="n">
         <v>0</v>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3360,9 +3240,6 @@
       <c r="M57" t="n">
         <v>0</v>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3410,9 +3287,6 @@
       <c r="M58" t="n">
         <v>0</v>
       </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3460,9 +3334,6 @@
       <c r="M59" t="n">
         <v>0</v>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3510,9 +3381,6 @@
       <c r="M60" t="n">
         <v>0</v>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3560,9 +3428,6 @@
       <c r="M61" t="n">
         <v>0</v>
       </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3610,9 +3475,6 @@
       <c r="M62" t="n">
         <v>0</v>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3660,9 +3522,6 @@
       <c r="M63" t="n">
         <v>0</v>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3710,9 +3569,6 @@
       <c r="M64" t="n">
         <v>0</v>
       </c>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3818,9 +3674,6 @@
       <c r="M66" t="n">
         <v>0</v>
       </c>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3868,9 +3721,6 @@
       <c r="M67" t="n">
         <v>0</v>
       </c>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3918,9 +3768,6 @@
       <c r="M68" t="n">
         <v>0</v>
       </c>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3968,9 +3815,6 @@
       <c r="M69" t="n">
         <v>0</v>
       </c>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4018,9 +3862,6 @@
       <c r="M70" t="n">
         <v>0</v>
       </c>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4068,9 +3909,6 @@
       <c r="M71" t="n">
         <v>0</v>
       </c>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4168,9 +4006,6 @@
       <c r="M73" t="n">
         <v>0</v>
       </c>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4218,9 +4053,6 @@
       <c r="M74" t="n">
         <v>0</v>
       </c>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4268,9 +4100,6 @@
       <c r="M75" t="n">
         <v>0</v>
       </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -4324,6 +4153,357 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unit type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Units on site</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Levelling</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Cleaning</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Demob</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Labour done now (install+steps+levelling+cleaning) x units</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Demob at demob x units</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Transport each way</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Delivery legs (done)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Pickup legs (at demob)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FWF</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>238</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.44</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>36.44</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8672.719999999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8672.719999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>11305</v>
+      </c>
+      <c r="L2" t="n">
+        <v>11305</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Accessible toilet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>88.48999999999999</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>88.48999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>353.96</v>
+      </c>
+      <c r="I3" t="n">
+        <v>353.96</v>
+      </c>
+      <c r="J3" t="n">
+        <v>500</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Toilet block 6 m (8 sewer-connected, 6 tank-mounted)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="D4" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="G4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7869.96</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2040.36</v>
+      </c>
+      <c r="J4" t="n">
+        <v>500</v>
+      </c>
+      <c r="K4" t="n">
+        <v>7000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>16-pan block</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="D5" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1124.28</v>
+      </c>
+      <c r="I5" t="n">
+        <v>291.48</v>
+      </c>
+      <c r="J5" t="n">
+        <v>500</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Waste tank 6 m</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="G6" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2435.94</v>
+      </c>
+      <c r="I6" t="n">
+        <v>874.4400000000001</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>no card line</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pee panel (WC09)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="G7" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2435.94</v>
+      </c>
+      <c r="I7" t="n">
+        <v>874.4400000000001</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>no card line</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr"/>
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="n">
+        <v>22892.8</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>13107.4</v>
+      </c>
+      <c r="J9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="n">
+        <v>21305</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>21305</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rates are the 2026 card per unit, ex GST. Baseplan line 144 charges blocks at $603.78 (install, steps, cleaning, demob) and leaves out levelling $104.10; the card has levelling on every block line. Waste tanks and pee panels have no transport line on the card; Baseplan charges none. Pee panel labour is the street card row 22, as authorised 9 Oct.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4767,7 +4947,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Toilets breakdown: no steps on the 16-pan blocks
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
@@ -4249,9 +4249,6 @@
       <c r="C2" t="n">
         <v>36.44</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>36.44</v>
       </c>
@@ -4283,9 +4280,6 @@
       <c r="C3" t="n">
         <v>88.48999999999999</v>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>88.48999999999999</v>
       </c>
@@ -4357,9 +4351,7 @@
       <c r="C5" t="n">
         <v>145.74</v>
       </c>
-      <c r="D5" t="n">
-        <v>156.15</v>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>104.1</v>
       </c>
@@ -4370,7 +4362,7 @@
         <v>145.74</v>
       </c>
       <c r="H5" t="n">
-        <v>1124.28</v>
+        <v>811.98</v>
       </c>
       <c r="I5" t="n">
         <v>291.48</v>
@@ -4397,7 +4389,6 @@
       <c r="C6" t="n">
         <v>145.74</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>104.1</v>
       </c>
@@ -4437,7 +4428,6 @@
       <c r="C7" t="n">
         <v>145.74</v>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>104.1</v>
       </c>
@@ -4465,6 +4455,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -4478,7 +4469,7 @@
       <c r="F9" s="1" t="inlineStr"/>
       <c r="G9" s="1" t="inlineStr"/>
       <c r="H9" s="1" t="n">
-        <v>22892.8</v>
+        <v>22580.5</v>
       </c>
       <c r="I9" s="1" t="n">
         <v>13107.4</v>
@@ -4491,10 +4482,11 @@
         <v>21305</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rates are the 2026 card per unit, ex GST. Baseplan line 144 charges blocks at $603.78 (install, steps, cleaning, demob) and leaves out levelling $104.10; the card has levelling on every block line. Waste tanks and pee panels have no transport line on the card; Baseplan charges none. Pee panel labour is the street card row 22, as authorised 9 Oct.</t>
+          <t>Rates are the 2026 card per unit, ex GST. Baseplan line 144 charges blocks at $603.78 (install, steps, cleaning, demob) and leaves out levelling $104.10; the card has levelling on every block line. Waste tanks and pee panels have no transport line on the card; Baseplan charges none. No steps on the 16-pan blocks (Andrew, 22 Oct). Pee panel labour is the street card row 22, as authorised 9 Oct.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Toilets: servicing breakdown by area and reference
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968955_Toilets_for_Branch_22Oct2026.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 by reference" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labour &amp; transport breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 charge lines" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9968955 charge lines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4351,7 +4352,6 @@
       <c r="C5" t="n">
         <v>145.74</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>104.1</v>
       </c>
@@ -4455,7 +4455,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -4482,7 +4481,6 @@
         <v>21305</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -4496,6 +4494,4647 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O94"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FWF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accessible</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>16-pan</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Waste tanks</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Sewer blocks</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tank-mounted blocks</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Pump-outs a night (FWF + accessible)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Tank pump-outs a night (tanks + 16-pan)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sewer cleans a night</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Pump-outs x 3 nights $</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Tank pump-outs x 3 $</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Sewer cleans x 3 $</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Total 3 nights $</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BJR01</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PG01</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PG03</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PG05</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PG29</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SVP01</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>T0162</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T0176</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>WC12</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>874.4400000000001</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>874.4400000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WC15</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1561.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1561.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>WC16</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1561.5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1561.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WC17</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1561.5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1561.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>WC43</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>10</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2186.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>WC73</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>1 Pit Lane, Paddock &amp; Teams subtotal</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="J16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="1" t="n">
+        <v>5465.25</v>
+      </c>
+      <c r="M16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="1" t="n">
+        <v>4684.5</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>10149.75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>WC19</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>WC20</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>3747.6</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>3747.6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WC21</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1311.66</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1311.66</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>WC44</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>WC86</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2 Island North / Freight subtotal</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr"/>
+      <c r="C22" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="1" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M22" s="1" t="n">
+        <v>3747.6</v>
+      </c>
+      <c r="N22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="1" t="n">
+        <v>5933.7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>T0024</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>WC04</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>WC05</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1873.8</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1873.8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>WC06</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>WC07</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>20</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>20</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>4372.2</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>4372.2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WC11</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>WC41</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>10</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>2186.1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>3 Island West — EVL, Race Admin &amp; Merch subtotal</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr"/>
+      <c r="C30" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="J30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1" t="n">
+        <v>8088.57</v>
+      </c>
+      <c r="M30" s="1" t="n">
+        <v>1873.8</v>
+      </c>
+      <c r="N30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1" t="n">
+        <v>9962.370000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>WC01</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>655.83</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>655.83</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>WC02</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>WC31</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M33" t="n">
+        <v>3747.6</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>3966.21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>WC34</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>WC38</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WC39</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>WC40</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>5</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1093.05</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1093.05</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>WC42</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>WC65</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>4 Commodore Park &amp; The Hill entry subtotal</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr"/>
+      <c r="C40" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="J40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="1" t="n">
+        <v>3497.76</v>
+      </c>
+      <c r="M40" s="1" t="n">
+        <v>3747.6</v>
+      </c>
+      <c r="N40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="1" t="n">
+        <v>7245.36</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>5 Median Strip — FOAM</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>WC09</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>10</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>1561.5</v>
+      </c>
+      <c r="O41" t="n">
+        <v>3747.6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>5 Median Strip — FOAM</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>WC10</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>655.83</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>655.83</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>5 Median Strip — FOAM</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>WC28</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>5 Median Strip — FOAM</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>WC29</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>7</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>7</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1530.27</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>1530.27</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>5 Median Strip — FOAM subtotal</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr"/>
+      <c r="C45" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="J45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" s="1" t="n">
+        <v>4590.81</v>
+      </c>
+      <c r="M45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="1" t="n">
+        <v>1561.5</v>
+      </c>
+      <c r="O45" s="1" t="n">
+        <v>6152.31</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>6 Main Beach Parade / Seaside North</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>WC27</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
+        <v>1873.8</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>1873.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>6 Main Beach Parade / Seaside North</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>WC33</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>17</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>17</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>3716.37</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
+        <v>3716.37</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>6 Main Beach Parade / Seaside North</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>WC60</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>3747.6</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>3747.6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>6 Main Beach Parade / Seaside North</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>WC61</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>8</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1748.88</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" t="n">
+        <v>1748.88</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>6 Main Beach Parade / Seaside North subtotal</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr"/>
+      <c r="C50" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I50" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="J50" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="1" t="n">
+        <v>5465.25</v>
+      </c>
+      <c r="M50" s="1" t="n">
+        <v>5621.4</v>
+      </c>
+      <c r="N50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="1" t="n">
+        <v>11086.65</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>WC23</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>5</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1093.05</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" t="n">
+        <v>1093.05</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>WC26</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>WC50</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>WC56</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>12</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>12</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2623.32</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
+        <v>2623.32</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>WC57</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>WC59</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>7</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1530.27</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>1530.27</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>7 Main Beach Seaside — Supply / North subtotal</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="J57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="1" t="n">
+        <v>6121.08</v>
+      </c>
+      <c r="M57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="1" t="n">
+        <v>6121.08</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>8 Main Beach Seaside — Mid</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>WC25</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>8 Main Beach Seaside — Mid</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>WC45</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>8</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>1748.88</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
+        <v>1748.88</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>8 Main Beach Seaside — Mid</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>WC47</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>1</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>8 Main Beach Seaside — Mid subtotal</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr"/>
+      <c r="C61" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="J61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="1" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="1" t="n">
+        <v>2186.1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SPASHDOWN</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>WC13</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>WC24</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>WC54</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>6</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
+        <v>1311.66</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" t="n">
+        <v>1311.66</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>WC55</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>9 Main Beach Seaside — Mid-South subtotal</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="inlineStr"/>
+      <c r="C67" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="J67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="1" t="n">
+        <v>2186.1</v>
+      </c>
+      <c r="M67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" s="1" t="n">
+        <v>2186.1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>WC46</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>WC48</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>4</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="n">
+        <v>874.4400000000001</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
+        <v>874.4400000000001</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>WC49</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>3</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>3</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
+        <v>655.83</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
+        <v>655.83</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>WC51</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>6</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>7</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
+        <v>1530.27</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>1530.27</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>WC53</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" t="n">
+        <v>3</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="n">
+        <v>655.83</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>655.83</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>10 Main Beach Seaside — South subtotal</t>
+        </is>
+      </c>
+      <c r="B73" s="1" t="inlineStr"/>
+      <c r="C73" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="D73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="J73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="1" t="n">
+        <v>3934.98</v>
+      </c>
+      <c r="M73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" s="1" t="n">
+        <v>3934.98</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>11 Surfers Paradise / Cypress (north)</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>WC30</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>8</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" t="n">
+        <v>8</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="n">
+        <v>1748.88</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>1748.88</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>11 Surfers Paradise / Cypress (north)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>WC35</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>11 Surfers Paradise / Cypress (north)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>WC62</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" t="n">
+        <v>2</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>11 Surfers Paradise / Cypress (north) subtotal</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="D77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="J77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="1" t="n">
+        <v>2404.71</v>
+      </c>
+      <c r="M77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" s="1" t="n">
+        <v>2404.71</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>WC67</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>4</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" t="n">
+        <v>4</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>874.4400000000001</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>874.4400000000001</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>WC68</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>WC69</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>12</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" t="n">
+        <v>12</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>2623.32</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>2623.32</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>WC70</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>WC71</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>8</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" t="n">
+        <v>8</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1748.88</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>1748.88</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>12 Helen Park</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>WC72</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>1</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>12 Helen Park subtotal</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="inlineStr"/>
+      <c r="C84" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="D84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="J84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="1" t="n">
+        <v>5902.47</v>
+      </c>
+      <c r="M84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" s="1" t="n">
+        <v>5902.47</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>13 Cypress / Surfers Paradise Blvd</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>WC81</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>1</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="inlineStr">
+        <is>
+          <t>13 Cypress / Surfers Paradise Blvd subtotal</t>
+        </is>
+      </c>
+      <c r="B86" s="1" t="inlineStr"/>
+      <c r="C86" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="1" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" s="1" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>14 Coates Compound (Seaway)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>WC85</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="n">
+        <v>1</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
+        <is>
+          <t>14 Coates Compound (Seaway) subtotal</t>
+        </is>
+      </c>
+      <c r="B88" s="1" t="inlineStr"/>
+      <c r="C88" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="1" t="n">
+        <v>218.61</v>
+      </c>
+      <c r="M88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" s="1" t="n">
+        <v>218.61</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>0 No location yet</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>WC100</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="n">
+        <v>2</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>0 No location yet subtotal</t>
+        </is>
+      </c>
+      <c r="B90" s="1" t="inlineStr"/>
+      <c r="C90" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="1" t="n">
+        <v>437.22</v>
+      </c>
+      <c r="M90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="1" t="n">
+        <v>437.22</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr"/>
+      <c r="C92" s="1" t="n">
+        <v>238</v>
+      </c>
+      <c r="D92" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E92" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="G92" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="H92" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I92" s="1" t="n">
+        <v>242</v>
+      </c>
+      <c r="J92" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K92" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L92" s="1" t="n">
+        <v>52903.62</v>
+      </c>
+      <c r="M92" s="1" t="n">
+        <v>14990.4</v>
+      </c>
+      <c r="N92" s="1" t="n">
+        <v>6246</v>
+      </c>
+      <c r="O92" s="1" t="n">
+        <v>74140.02</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Rates: pump-out FWF or accessible $72.87 a service, tank pump-out and clean $624.6, sewer-connect clean and restock $260.25. Three services a unit: Fri 23, Sat 24, Sun 25 Oct nights. The 16-pan blocks are pumped as tanks and cleaned with the pump-out. Tank-mounted blocks are cleaned under the tank pump-out. Invoice from the tracker ticks after each night.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4939,7 +9578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>